<commit_message>
Excel DM rewrite: embed site link, no upfront price, IG delivery + office-visit close
</commit_message>
<xml_diff>
--- a/KB_Rewaq_Leads.xlsx
+++ b/KB_Rewaq_Leads.xlsx
@@ -488,7 +488,7 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="52" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -525,7 +525,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Ready DM Message (copy/paste)</t>
+          <t>Ready DM Message (link inside)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -534,7 +534,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="78" customHeight="1">
+    <row r="2" ht="140" customHeight="1">
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
@@ -565,7 +565,15 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Hi Midyaf! I built a FREE sample 3D website for your salon (link inside). KB Rewaq Digital makes salon sites + Instagram in 3 days, from 25 KWD. Want it with YOUR name? Reply YES.</t>
+          <t>Hi Midyaf Beauty Salon! 👋 Your salon deserves to be seen online.
+I'm Faizan from KB Rewaq Digital. I built a FREE sample website for your salon so you can see exactly what you'd get — no cost, no obligation.
+Here's what we do for salons like yours:
+🌐 Custom website — your name, services &amp; prices, online booking, Arabic + English
+📸 Instagram growth — you send us photos, we design your posts, reels &amp; stories and handle the posting, so your salon stays active and pulls in new clients
+📈 More visibility, more bookings — that's the whole point
+If you like the demo, I'll visit your salon for a free 15-minute overview and show you the full plan — no pressure, just a clear next step.
+Reply YES and I'll set it up. 🙌
+👉 Your free demo: https://faizanbashar215.github.io/kb-rewaq-digital/midyaf/</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -574,7 +582,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="78" customHeight="1">
+    <row r="3" ht="140" customHeight="1">
       <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
@@ -605,7 +613,15 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Hello Look Noor! Your competitors are online, you should be too. I made a free demo site for you (link inside). Professional salon website + social from 25 KWD, ready in 3 days. Interested?</t>
+          <t>Hello Look Noor Ladies! 👋 Your clients are already on Instagram — let's meet them there.
+I'm Faizan from KB Rewaq Digital. I built a FREE sample website for your salon so you can see exactly what you'd get — no cost, no obligation.
+Here's what we do for salons like yours:
+🌐 Custom website — your name, services &amp; prices, online booking, Arabic + English
+📸 Instagram growth — you send us photos, we design your posts, reels &amp; stories and handle the posting, so your salon stays active and pulls in new clients
+📈 More visibility, more bookings — that's the whole point
+If you like the demo, I'll visit your salon for a free 15-minute overview and show you the full plan — no pressure, just a clear next step.
+Reply YES and I'll set it up. 🙌
+👉 Your free demo: https://faizanbashar215.github.io/kb-rewaq-digital/looknoor/</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -614,7 +630,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="78" customHeight="1">
+    <row r="4" ht="140" customHeight="1">
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
@@ -645,7 +661,15 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Hi Monya Salon! Summer offers are great but a website brings more clients. I built you a free sample 3D site (link inside). Sites + Instagram from 25 KWD, 3-day delivery. Want it?</t>
+          <t>Hi Monya Ladies Salon! 👋 Summer is busy — a website catches the walk-ins you're missing.
+I'm Faizan from KB Rewaq Digital. I built a FREE sample website for your salon so you can see exactly what you'd get — no cost, no obligation.
+Here's what we do for salons like yours:
+🌐 Custom website — your name, services &amp; prices, online booking, Arabic + English
+📸 Instagram growth — you send us photos, we design your posts, reels &amp; stories and handle the posting, so your salon stays active and pulls in new clients
+📈 More visibility, more bookings — that's the whole point
+If you like the demo, I'll visit your salon for a free 15-minute overview and show you the full plan — no pressure, just a clear next step.
+Reply YES and I'll set it up. 🙌
+👉 Your free demo: https://faizanbashar215.github.io/kb-rewaq-digital/monya/</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -654,7 +678,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="78" customHeight="1">
+    <row r="5" ht="140" customHeight="1">
       <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
@@ -685,7 +709,15 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Hello Royal Jasmine! A royal salon deserves a royal website. I made one for you free (link inside). KB Rewaq Digital: site + social from 25 KWD, 3 days. Reply YES for your branded version.</t>
+          <t>Hello Royal Jasmine! 👋 A royal salon needs a royal presence online.
+I'm Faizan from KB Rewaq Digital. I built a FREE sample website for your salon so you can see exactly what you'd get — no cost, no obligation.
+Here's what we do for salons like yours:
+🌐 Custom website — your name, services &amp; prices, online booking, Arabic + English
+📸 Instagram growth — you send us photos, we design your posts, reels &amp; stories and handle the posting, so your salon stays active and pulls in new clients
+📈 More visibility, more bookings — that's the whole point
+If you like the demo, I'll visit your salon for a free 15-minute overview and show you the full plan — no pressure, just a clear next step.
+Reply YES and I'll set it up. 🙌
+👉 Your free demo: https://faizanbashar215.github.io/kb-rewaq-digital/royaljasmine/</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -694,7 +726,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="78" customHeight="1">
+    <row r="6" ht="140" customHeight="1">
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
@@ -725,7 +757,15 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Hi Larene! Your spa needs a beautiful site to match. I built a free 3D demo (link inside). We do salon/spa websites + Instagram from 25 KWD, ready in 3 days. Interested?</t>
+          <t>Hi Larene Beauty Spa! 👋 Your spa should look as beautiful online as it does inside.
+I'm Faizan from KB Rewaq Digital. I built a FREE sample website for your salon so you can see exactly what you'd get — no cost, no obligation.
+Here's what we do for salons like yours:
+🌐 Custom website — your name, services &amp; prices, online booking, Arabic + English
+📸 Instagram growth — you send us photos, we design your posts, reels &amp; stories and handle the posting, so your salon stays active and pulls in new clients
+📈 More visibility, more bookings — that's the whole point
+If you like the demo, I'll visit your salon for a free 15-minute overview and show you the full plan — no pressure, just a clear next step.
+Reply YES and I'll set it up. 🙌
+👉 Your free demo: https://faizanbashar215.github.io/kb-rewaq-digital/larene/</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -777,7 +817,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>1. Click the GREEN phone cell -&gt; opens WhatsApp to that lead with your DM pre-typed.</t>
+          <t>1. Click the GREEN phone cell -&gt; opens WhatsApp to that lead with your DM + their demo link pre-typed.</t>
         </is>
       </c>
     </row>
@@ -791,21 +831,21 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>3. Send the DM on WhatsApp. When they reply, change Status column to: replied / won / paid.</t>
+          <t>3. Send the DM on WhatsApp. The link is already inside the message.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>4. Demo sites are LIVE on GitHub Pages -&gt; the prospect can open &amp; see them too.</t>
+          <t>4. When they reply YES, visit their salon for a free overview, then discuss price &amp; sign up.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>5. After sending, mark Status and we track weekly conversion.</t>
+          <t>5. After sending, change Status to: replied / won / paid.</t>
         </is>
       </c>
     </row>

</xml_diff>